<commit_message>
Updated validator with for
</commit_message>
<xml_diff>
--- a/docs/lab03/Lab03_WBT_TCs_Form.xlsx
+++ b/docs/lab03/Lab03_WBT_TCs_Form.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10313"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34340B63-9519-4A9D-B3B1-55B743C940D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A0BB40A-0174-FB44-BE76-C85696C54D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Statement" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="130">
   <si>
     <t>VVSS, Info Romana, 2025-2026</t>
   </si>
@@ -424,36 +424,12 @@
     <t>1. Evidenţa bauturilor din colecţia personală</t>
   </si>
   <si>
-    <t>String errors = ""</t>
-  </si>
-  <si>
     <t>Req02_L10</t>
   </si>
   <si>
     <t>Req02_L12</t>
   </si>
   <si>
-    <t>if (item.getProduct().getId() &lt;= 0)</t>
-  </si>
-  <si>
-    <t>errors += "Product ID invalid!\n";</t>
-  </si>
-  <si>
-    <t>if (item.getQuantity() &lt;= 0)</t>
-  </si>
-  <si>
-    <t>errors += "Cantitate invalida!\n";</t>
-  </si>
-  <si>
-    <t>if (!errors.isEmpty())</t>
-  </si>
-  <si>
-    <t>throw new ValidationException(errors);</t>
-  </si>
-  <si>
-    <t>// Iesire normala (metoda se termina)</t>
-  </si>
-  <si>
     <t>Req02_L13</t>
   </si>
   <si>
@@ -472,18 +448,6 @@
     <t>Req02_L20</t>
   </si>
   <si>
-    <t>1 - 2(F) - 4(F) - 6(F) - 8</t>
-  </si>
-  <si>
-    <t>1 - 2(T) - 3 - 4(F) - 6(T) - 7 - 8</t>
-  </si>
-  <si>
-    <t>1 - 2(F) - 4(T) - 5 - 6(T) - 7 - 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 - 2(T) - 3 - 4(T) - t - 6(T) - 7 - 8 </t>
-  </si>
-  <si>
     <t>F02_P04</t>
   </si>
   <si>
@@ -532,18 +496,6 @@
     <t>F02_Cond03 !errors.isEmpty()</t>
   </si>
   <si>
-    <t>1, 2, 4, 6, 8</t>
-  </si>
-  <si>
-    <t>1, 2, 3, 4, 6, 7</t>
-  </si>
-  <si>
-    <t>1, 2, 4, 5, 6, 7</t>
-  </si>
-  <si>
-    <t>1, 2, 3, 4, 5, 6, 7</t>
-  </si>
-  <si>
     <t>X</t>
   </si>
   <si>
@@ -563,13 +515,73 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>StringBuilder errors = new StringBuilder();</t>
+  </si>
+  <si>
+    <t>Map&lt;Boolean, String&gt; checks = Map.of(</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    item.getProduct().getId() &lt;= 0, "Product ID invalid!\n",</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    item.getQuantity() &lt;= 0, "Cantitate invalida!\n");</t>
+  </si>
+  <si>
+    <t>for (Map.Entry&lt;Boolean, String&gt; check : checks.entrySet()) {</t>
+  </si>
+  <si>
+    <t>if (check.getKey()) {</t>
+  </si>
+  <si>
+    <t>errors.append(check.getValue()); } }</t>
+  </si>
+  <si>
+    <t>if (!errors.isEmpty())\</t>
+  </si>
+  <si>
+    <t>Req02_L21</t>
+  </si>
+  <si>
+    <t>Req02_L22</t>
+  </si>
+  <si>
+    <t>throw new ValidationException(errors.toString());</t>
+  </si>
+  <si>
+    <t>// Iesire normala</t>
+  </si>
+  <si>
+    <t>1→2→3(T)→4→2→3(F)→2→5(T)→6</t>
+  </si>
+  <si>
+    <t>1→2→3(F)→2→3(T)→4→2→5(T)→6</t>
+  </si>
+  <si>
+    <t>1→2→3(T)→4→2→3(T)→4→2→5(T)→6</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 2, 3, 2, 5, 7</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 4, 2, 3, 2, 5, 6</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 2, 3, 4, 2, 5, 6</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 4, 2, 3, 4, 2, 5, 6</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 5, 2, 3, 5, 2, 7, 9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1234,7 +1246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1316,235 +1328,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1558,10 +1342,213 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1583,23 +1570,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>651933</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>16934</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>95489</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>105038</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>766233</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>139701</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>187380</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>76391</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B12BB563-7EC7-1048-8757-6FF3C1A5E892}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{994AA24C-0821-F345-B697-897E0C4CEE65}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1615,8 +1602,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="651933" y="3132667"/>
-          <a:ext cx="2882900" cy="1485900"/>
+          <a:off x="763910" y="3733609"/>
+          <a:ext cx="4026026" cy="2645038"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1627,23 +1614,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>160867</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>8467</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>630225</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>171879</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>334433</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>42334</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>257819</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>155306</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="7" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E58122DB-00DA-D84D-B0B6-4A153B89C321}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28A5C19F-EEDE-9F41-8E61-88020E33A194}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1659,8 +1646,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6832600" y="1761067"/>
-          <a:ext cx="2882900" cy="7239000"/>
+          <a:off x="5901202" y="1699699"/>
+          <a:ext cx="4974963" cy="6094705"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1673,9 +1660,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1713,9 +1700,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1748,9 +1735,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1783,9 +1787,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1963,26 +1984,26 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:P20"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="15" max="15" width="19.46484375" customWidth="1"/>
+    <col min="15" max="15" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B1" s="8"/>
-      <c r="D1" s="61" t="s">
+      <c r="D1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="63"/>
-    </row>
-    <row r="2" spans="2:16">
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="46"/>
+    </row>
+    <row r="2" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B2" s="29" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:16">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1992,7 +2013,7 @@
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
     </row>
-    <row r="5" spans="2:16">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
@@ -2002,7 +2023,7 @@
       <c r="O5" s="26"/>
       <c r="P5" s="26"/>
     </row>
-    <row r="6" spans="2:16">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
@@ -2014,7 +2035,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:16">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2029,7 +2050,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="8" spans="2:16">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -2044,7 +2065,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="9" spans="2:16">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>78</v>
       </c>
@@ -2061,7 +2082,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="10" spans="2:16">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>73</v>
       </c>
@@ -2069,7 +2090,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="2:16">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B11" s="30" t="s">
         <v>77</v>
       </c>
@@ -2077,15 +2098,15 @@
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="2:16">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.2">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B20" s="1"/>
     </row>
   </sheetData>
@@ -2103,410 +2124,432 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:T26"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="17" max="17" width="10.46484375" customWidth="1"/>
+    <col min="17" max="17" width="10.5" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20">
+    <row r="1" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B1" s="8"/>
-      <c r="D1" s="61" t="s">
+      <c r="D1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="63"/>
-    </row>
-    <row r="3" spans="2:20">
-      <c r="B3" s="79" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="46"/>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B3" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="81"/>
-    </row>
-    <row r="6" spans="2:20">
-      <c r="B6" s="61" t="s">
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="50"/>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="63"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="46"/>
       <c r="F6" s="22"/>
       <c r="G6" s="22"/>
-      <c r="I6" s="61" t="s">
+      <c r="I6" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="62"/>
-      <c r="K6" s="62"/>
-      <c r="L6" s="62"/>
-      <c r="M6" s="62"/>
-      <c r="N6" s="62"/>
-      <c r="O6" s="62"/>
-      <c r="Q6" s="61" t="s">
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="45"/>
+      <c r="M6" s="45"/>
+      <c r="N6" s="45"/>
+      <c r="O6" s="45"/>
+      <c r="Q6" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="R6" s="62"/>
-      <c r="S6" s="62"/>
-      <c r="T6" s="62"/>
-    </row>
-    <row r="8" spans="2:20">
+      <c r="R6" s="45"/>
+      <c r="S6" s="45"/>
+      <c r="T6" s="45"/>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B8" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="91" t="s">
+      <c r="C8" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
       <c r="F8" s="24"/>
       <c r="G8" s="24"/>
       <c r="I8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="Q8" s="75" t="s">
+      <c r="Q8" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="R8" s="75"/>
-      <c r="S8" s="75"/>
+      <c r="R8" s="61"/>
+      <c r="S8" s="61"/>
       <c r="T8" s="25">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="2:20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B9" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" s="74" t="s">
         <v>79</v>
       </c>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
+      <c r="C9" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" s="51"/>
+      <c r="E9" s="51"/>
       <c r="F9" s="27"/>
       <c r="G9" s="27"/>
       <c r="I9" s="28"/>
-      <c r="Q9" s="75" t="s">
+      <c r="Q9" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="R9" s="75"/>
-      <c r="S9" s="75"/>
+      <c r="R9" s="61"/>
+      <c r="S9" s="61"/>
       <c r="T9" s="25">
-        <f>10-8+2</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="2:20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B10" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="74" t="s">
-        <v>82</v>
-      </c>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
+        <v>80</v>
+      </c>
+      <c r="C10" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
       <c r="F10" s="27"/>
       <c r="G10" s="27"/>
-      <c r="I10" s="82"/>
-      <c r="J10" s="83"/>
-      <c r="K10" s="83"/>
-      <c r="L10" s="83"/>
-      <c r="M10" s="83"/>
-      <c r="N10" s="83"/>
-      <c r="O10" s="84"/>
-      <c r="Q10" s="75" t="s">
+      <c r="I10" s="52"/>
+      <c r="J10" s="53"/>
+      <c r="K10" s="53"/>
+      <c r="L10" s="53"/>
+      <c r="M10" s="53"/>
+      <c r="N10" s="53"/>
+      <c r="O10" s="54"/>
+      <c r="Q10" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="R10" s="75" t="s">
+      <c r="R10" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="S10" s="75"/>
+      <c r="S10" s="61"/>
       <c r="T10" s="25">
-        <f>3+1</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="2:20">
+        <f>5</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B11" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="C11" s="74" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11" s="74"/>
-      <c r="E11" s="74"/>
+        <v>81</v>
+      </c>
+      <c r="C11" s="51" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" s="51"/>
+      <c r="E11" s="51"/>
       <c r="F11" s="27"/>
       <c r="G11" s="27"/>
-      <c r="I11" s="85"/>
-      <c r="J11" s="86"/>
-      <c r="K11" s="86"/>
-      <c r="L11" s="86"/>
-      <c r="M11" s="86"/>
-      <c r="N11" s="86"/>
-      <c r="O11" s="87"/>
-    </row>
-    <row r="12" spans="2:20">
+      <c r="I11" s="55"/>
+      <c r="J11" s="56"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="56"/>
+      <c r="N11" s="56"/>
+      <c r="O11" s="57"/>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B12" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="C12" s="74" t="s">
-        <v>84</v>
-      </c>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
+        <v>82</v>
+      </c>
+      <c r="C12" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="51"/>
+      <c r="E12" s="51"/>
       <c r="F12" s="27"/>
       <c r="G12" s="27"/>
-      <c r="I12" s="85"/>
-      <c r="J12" s="86"/>
-      <c r="K12" s="86"/>
-      <c r="L12" s="86"/>
-      <c r="M12" s="86"/>
-      <c r="N12" s="86"/>
-      <c r="O12" s="87"/>
-    </row>
-    <row r="13" spans="2:20">
+      <c r="I12" s="55"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="56"/>
+      <c r="L12" s="56"/>
+      <c r="M12" s="56"/>
+      <c r="N12" s="56"/>
+      <c r="O12" s="57"/>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B13" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="C13" s="76" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="76"/>
-      <c r="E13" s="76"/>
+        <v>83</v>
+      </c>
+      <c r="C13" s="63" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="63"/>
+      <c r="E13" s="63"/>
       <c r="F13" s="27"/>
       <c r="G13" s="27"/>
-      <c r="I13" s="85"/>
-      <c r="J13" s="86"/>
-      <c r="K13" s="86"/>
-      <c r="L13" s="86"/>
-      <c r="M13" s="86"/>
-      <c r="N13" s="86"/>
-      <c r="O13" s="87"/>
-      <c r="Q13" s="61" t="s">
+      <c r="I13" s="55"/>
+      <c r="J13" s="56"/>
+      <c r="K13" s="56"/>
+      <c r="L13" s="56"/>
+      <c r="M13" s="56"/>
+      <c r="N13" s="56"/>
+      <c r="O13" s="57"/>
+      <c r="Q13" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="R13" s="62"/>
-      <c r="S13" s="62"/>
-      <c r="T13" s="62"/>
-    </row>
-    <row r="14" spans="2:20">
+      <c r="R13" s="45"/>
+      <c r="S13" s="45"/>
+      <c r="T13" s="45"/>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B14" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="C14" s="78" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" s="78"/>
-      <c r="E14" s="78"/>
+        <v>85</v>
+      </c>
+      <c r="C14" s="65" t="s">
+        <v>115</v>
+      </c>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
       <c r="F14" s="27"/>
       <c r="G14" s="27"/>
-      <c r="I14" s="85"/>
-      <c r="J14" s="86"/>
-      <c r="K14" s="86"/>
-      <c r="L14" s="86"/>
-      <c r="M14" s="86"/>
-      <c r="N14" s="86"/>
-      <c r="O14" s="87"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="56"/>
+      <c r="K14" s="56"/>
+      <c r="L14" s="56"/>
+      <c r="M14" s="56"/>
+      <c r="N14" s="56"/>
+      <c r="O14" s="57"/>
       <c r="Q14" s="22"/>
       <c r="R14" s="22"/>
       <c r="S14" s="22"/>
       <c r="T14" s="22"/>
     </row>
-    <row r="15" spans="2:20">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B15" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="77" t="s">
-        <v>87</v>
-      </c>
-      <c r="D15" s="77"/>
-      <c r="E15" s="77"/>
+        <v>84</v>
+      </c>
+      <c r="C15" s="64" t="s">
+        <v>116</v>
+      </c>
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
       <c r="F15" s="27"/>
       <c r="G15" s="27"/>
-      <c r="I15" s="85"/>
-      <c r="J15" s="86"/>
-      <c r="K15" s="86"/>
-      <c r="L15" s="86"/>
-      <c r="M15" s="86"/>
-      <c r="N15" s="86"/>
-      <c r="O15" s="87"/>
-    </row>
-    <row r="16" spans="2:20">
+      <c r="I15" s="55"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="56"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="56"/>
+      <c r="O15" s="57"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B16" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="C16" s="77" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="77"/>
-      <c r="E16" s="77"/>
+        <v>86</v>
+      </c>
+      <c r="C16" s="64" t="s">
+        <v>117</v>
+      </c>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
       <c r="F16" s="27"/>
       <c r="G16" s="27"/>
-      <c r="I16" s="85"/>
-      <c r="J16" s="86"/>
-      <c r="K16" s="86"/>
-      <c r="L16" s="86"/>
-      <c r="M16" s="86"/>
-      <c r="N16" s="86"/>
-      <c r="O16" s="87"/>
-    </row>
-    <row r="17" spans="9:20">
-      <c r="I17" s="85"/>
-      <c r="J17" s="86"/>
-      <c r="K17" s="86"/>
-      <c r="L17" s="86"/>
-      <c r="M17" s="86"/>
-      <c r="N17" s="86"/>
-      <c r="O17" s="87"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="56"/>
+      <c r="K16" s="56"/>
+      <c r="L16" s="56"/>
+      <c r="M16" s="56"/>
+      <c r="N16" s="56"/>
+      <c r="O16" s="57"/>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B17" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" t="s">
+        <v>120</v>
+      </c>
+      <c r="I17" s="55"/>
+      <c r="J17" s="56"/>
+      <c r="K17" s="56"/>
+      <c r="L17" s="56"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="56"/>
+      <c r="O17" s="57"/>
       <c r="Q17" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="R17" s="91" t="s">
+      <c r="R17" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="S17" s="91"/>
-      <c r="T17" s="91"/>
-    </row>
-    <row r="18" spans="9:20">
-      <c r="I18" s="85"/>
-      <c r="J18" s="86"/>
-      <c r="K18" s="86"/>
-      <c r="L18" s="86"/>
-      <c r="M18" s="86"/>
-      <c r="N18" s="86"/>
-      <c r="O18" s="87"/>
+      <c r="S17" s="62"/>
+      <c r="T17" s="62"/>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B18" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" t="s">
+        <v>121</v>
+      </c>
+      <c r="I18" s="55"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="56"/>
+      <c r="M18" s="56"/>
+      <c r="N18" s="56"/>
+      <c r="O18" s="57"/>
       <c r="Q18" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="R18" s="73" t="s">
-        <v>95</v>
-      </c>
-      <c r="S18" s="73"/>
-      <c r="T18" s="73"/>
-    </row>
-    <row r="19" spans="9:20">
-      <c r="I19" s="85"/>
-      <c r="J19" s="86"/>
-      <c r="K19" s="86"/>
-      <c r="L19" s="86"/>
-      <c r="M19" s="86"/>
-      <c r="N19" s="86"/>
-      <c r="O19" s="87"/>
+      <c r="R18" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="S18" s="47"/>
+      <c r="T18" s="47"/>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I19" s="55"/>
+      <c r="J19" s="56"/>
+      <c r="K19" s="56"/>
+      <c r="L19" s="56"/>
+      <c r="M19" s="56"/>
+      <c r="N19" s="56"/>
+      <c r="O19" s="57"/>
       <c r="Q19" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="R19" s="73" t="s">
-        <v>96</v>
-      </c>
-      <c r="S19" s="73"/>
-      <c r="T19" s="73"/>
-    </row>
-    <row r="20" spans="9:20">
-      <c r="I20" s="85"/>
-      <c r="J20" s="86"/>
-      <c r="K20" s="86"/>
-      <c r="L20" s="86"/>
-      <c r="M20" s="86"/>
-      <c r="N20" s="86"/>
-      <c r="O20" s="87"/>
+      <c r="R19" s="47" t="s">
+        <v>122</v>
+      </c>
+      <c r="S19" s="47"/>
+      <c r="T19" s="47"/>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I20" s="55"/>
+      <c r="J20" s="56"/>
+      <c r="K20" s="56"/>
+      <c r="L20" s="56"/>
+      <c r="M20" s="56"/>
+      <c r="N20" s="56"/>
+      <c r="O20" s="57"/>
       <c r="Q20" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="R20" s="73" t="s">
-        <v>97</v>
-      </c>
-      <c r="S20" s="73"/>
-      <c r="T20" s="73"/>
-    </row>
-    <row r="21" spans="9:20">
-      <c r="I21" s="85"/>
-      <c r="J21" s="86"/>
-      <c r="K21" s="86"/>
-      <c r="L21" s="86"/>
-      <c r="M21" s="86"/>
-      <c r="N21" s="86"/>
-      <c r="O21" s="87"/>
+      <c r="R20" s="47" t="s">
+        <v>123</v>
+      </c>
+      <c r="S20" s="47"/>
+      <c r="T20" s="47"/>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I21" s="55"/>
+      <c r="J21" s="56"/>
+      <c r="K21" s="56"/>
+      <c r="L21" s="56"/>
+      <c r="M21" s="56"/>
+      <c r="N21" s="56"/>
+      <c r="O21" s="57"/>
       <c r="Q21" s="26" t="s">
-        <v>99</v>
-      </c>
-      <c r="R21" s="73" t="s">
-        <v>98</v>
-      </c>
-      <c r="S21" s="73"/>
-      <c r="T21" s="73"/>
-    </row>
-    <row r="22" spans="9:20">
-      <c r="I22" s="85"/>
-      <c r="J22" s="86"/>
-      <c r="K22" s="86"/>
-      <c r="L22" s="86"/>
-      <c r="M22" s="86"/>
-      <c r="N22" s="86"/>
-      <c r="O22" s="87"/>
+        <v>87</v>
+      </c>
+      <c r="R21" s="47" t="s">
+        <v>124</v>
+      </c>
+      <c r="S21" s="47"/>
+      <c r="T21" s="47"/>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I22" s="55"/>
+      <c r="J22" s="56"/>
+      <c r="K22" s="56"/>
+      <c r="L22" s="56"/>
+      <c r="M22" s="56"/>
+      <c r="N22" s="56"/>
+      <c r="O22" s="57"/>
       <c r="Q22" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="R22" s="73" t="s">
+      <c r="R22" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="S22" s="73"/>
-      <c r="T22" s="73"/>
-    </row>
-    <row r="23" spans="9:20">
-      <c r="I23" s="85"/>
-      <c r="J23" s="86"/>
-      <c r="K23" s="86"/>
-      <c r="L23" s="86"/>
-      <c r="M23" s="86"/>
-      <c r="N23" s="86"/>
-      <c r="O23" s="87"/>
+      <c r="S22" s="47"/>
+      <c r="T22" s="47"/>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I23" s="55"/>
+      <c r="J23" s="56"/>
+      <c r="K23" s="56"/>
+      <c r="L23" s="56"/>
+      <c r="M23" s="56"/>
+      <c r="N23" s="56"/>
+      <c r="O23" s="57"/>
       <c r="Q23" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="R23" s="73" t="s">
+      <c r="R23" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="S23" s="73"/>
-      <c r="T23" s="73"/>
-    </row>
-    <row r="24" spans="9:20">
-      <c r="I24" s="85"/>
-      <c r="J24" s="86"/>
-      <c r="K24" s="86"/>
-      <c r="L24" s="86"/>
-      <c r="M24" s="86"/>
-      <c r="N24" s="86"/>
-      <c r="O24" s="87"/>
-    </row>
-    <row r="25" spans="9:20">
-      <c r="I25" s="85"/>
-      <c r="J25" s="86"/>
-      <c r="K25" s="86"/>
-      <c r="L25" s="86"/>
-      <c r="M25" s="86"/>
-      <c r="N25" s="86"/>
-      <c r="O25" s="87"/>
-    </row>
-    <row r="26" spans="9:20">
-      <c r="I26" s="88"/>
-      <c r="J26" s="89"/>
-      <c r="K26" s="89"/>
-      <c r="L26" s="89"/>
-      <c r="M26" s="89"/>
-      <c r="N26" s="89"/>
-      <c r="O26" s="90"/>
+      <c r="S23" s="47"/>
+      <c r="T23" s="47"/>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I24" s="55"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="56"/>
+      <c r="L24" s="56"/>
+      <c r="M24" s="56"/>
+      <c r="N24" s="56"/>
+      <c r="O24" s="57"/>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I25" s="55"/>
+      <c r="J25" s="56"/>
+      <c r="K25" s="56"/>
+      <c r="L25" s="56"/>
+      <c r="M25" s="56"/>
+      <c r="N25" s="56"/>
+      <c r="O25" s="57"/>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="I26" s="58"/>
+      <c r="J26" s="59"/>
+      <c r="K26" s="59"/>
+      <c r="L26" s="59"/>
+      <c r="M26" s="59"/>
+      <c r="N26" s="59"/>
+      <c r="O26" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="R20:T20"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="Q9:S9"/>
+    <mergeCell ref="R18:T18"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="Q13:T13"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C16:E16"/>
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="R22:T22"/>
     <mergeCell ref="R23:T23"/>
@@ -2523,16 +2566,6 @@
     <mergeCell ref="Q6:T6"/>
     <mergeCell ref="R19:T19"/>
     <mergeCell ref="R21:T21"/>
-    <mergeCell ref="R20:T20"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="Q9:S9"/>
-    <mergeCell ref="R18:T18"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="Q13:T13"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C16:E16"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2547,169 +2580,169 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:V16"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12.33203125" customWidth="1"/>
-    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
-    <col min="5" max="5" width="19.796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.1328125" customWidth="1"/>
-    <col min="7" max="7" width="11.46484375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.1640625" customWidth="1"/>
+    <col min="7" max="7" width="11.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.33203125" customWidth="1"/>
     <col min="9" max="9" width="9.33203125" customWidth="1"/>
     <col min="10" max="10" width="26.33203125" customWidth="1"/>
-    <col min="11" max="11" width="6.1328125" customWidth="1"/>
-    <col min="12" max="13" width="8.796875" customWidth="1"/>
-    <col min="16" max="18" width="2.1328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="3.46484375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="2.1328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="4.1328125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.1328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.1640625" customWidth="1"/>
+    <col min="12" max="13" width="8.83203125" customWidth="1"/>
+    <col min="16" max="18" width="2.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="2.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22">
+    <row r="1" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B1" s="8"/>
-      <c r="D1" s="61" t="s">
+      <c r="D1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="63"/>
-    </row>
-    <row r="3" spans="2:22">
-      <c r="B3" s="79" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="46"/>
+    </row>
+    <row r="3" spans="2:22" x14ac:dyDescent="0.2">
+      <c r="B3" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="81"/>
-    </row>
-    <row r="5" spans="2:22">
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="50"/>
+    </row>
+    <row r="5" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B5" s="7"/>
     </row>
-    <row r="6" spans="2:22" ht="15.75">
-      <c r="B6" s="98" t="s">
+    <row r="6" spans="2:22" ht="16" x14ac:dyDescent="0.2">
+      <c r="B6" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="98" t="s">
+      <c r="C6" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="99" t="s">
+      <c r="D6" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="98" t="s">
+      <c r="E6" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="98"/>
-      <c r="G6" s="98"/>
-      <c r="H6" s="98"/>
-      <c r="I6" s="98"/>
-      <c r="J6" s="98"/>
-      <c r="K6" s="98"/>
-      <c r="L6" s="98"/>
-      <c r="M6" s="98"/>
-      <c r="N6" s="98"/>
-      <c r="O6" s="98"/>
-      <c r="P6" s="98"/>
-      <c r="Q6" s="98"/>
-      <c r="R6" s="98"/>
-      <c r="S6" s="98"/>
-      <c r="T6" s="98"/>
-      <c r="U6" s="98"/>
-      <c r="V6" s="98"/>
-    </row>
-    <row r="7" spans="2:22" ht="15.75">
-      <c r="B7" s="98"/>
-      <c r="C7" s="98"/>
-      <c r="D7" s="100"/>
-      <c r="E7" s="94" t="s">
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66"/>
+      <c r="K6" s="66"/>
+      <c r="L6" s="66"/>
+      <c r="M6" s="66"/>
+      <c r="N6" s="66"/>
+      <c r="O6" s="66"/>
+      <c r="P6" s="66"/>
+      <c r="Q6" s="66"/>
+      <c r="R6" s="66"/>
+      <c r="S6" s="66"/>
+      <c r="T6" s="66"/>
+      <c r="U6" s="66"/>
+      <c r="V6" s="66"/>
+    </row>
+    <row r="7" spans="2:22" ht="16" x14ac:dyDescent="0.2">
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="74" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="95" t="s">
+      <c r="F7" s="72" t="s">
         <v>36</v>
       </c>
-      <c r="G7" s="95"/>
-      <c r="H7" s="95"/>
-      <c r="I7" s="95"/>
-      <c r="J7" s="95"/>
-      <c r="K7" s="95"/>
-      <c r="L7" s="96" t="s">
+      <c r="G7" s="72"/>
+      <c r="H7" s="72"/>
+      <c r="I7" s="72"/>
+      <c r="J7" s="72"/>
+      <c r="K7" s="72"/>
+      <c r="L7" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="M7" s="96"/>
-      <c r="N7" s="96"/>
-      <c r="O7" s="96"/>
-      <c r="P7" s="97" t="s">
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="73"/>
+      <c r="P7" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="Q7" s="97"/>
-      <c r="R7" s="97"/>
-      <c r="S7" s="97"/>
-      <c r="T7" s="97"/>
-      <c r="U7" s="97"/>
-      <c r="V7" s="97"/>
-    </row>
-    <row r="8" spans="2:22" ht="15.5" customHeight="1">
-      <c r="B8" s="98"/>
-      <c r="C8" s="92" t="s">
+      <c r="Q7" s="69"/>
+      <c r="R7" s="69"/>
+      <c r="S7" s="69"/>
+      <c r="T7" s="69"/>
+      <c r="U7" s="69"/>
+      <c r="V7" s="69"/>
+    </row>
+    <row r="8" spans="2:22" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="66"/>
+      <c r="C8" s="70" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="70" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="74"/>
+      <c r="F8" s="72" t="s">
         <v>100</v>
       </c>
-      <c r="D8" s="92" t="s">
+      <c r="G8" s="72"/>
+      <c r="H8" s="72" t="s">
         <v>101</v>
       </c>
-      <c r="E8" s="94"/>
-      <c r="F8" s="95" t="s">
-        <v>112</v>
-      </c>
-      <c r="G8" s="95"/>
-      <c r="H8" s="95" t="s">
-        <v>113</v>
-      </c>
-      <c r="I8" s="95"/>
-      <c r="J8" s="95" t="s">
-        <v>114</v>
-      </c>
-      <c r="K8" s="95"/>
-      <c r="L8" s="96" t="s">
+      <c r="I8" s="72"/>
+      <c r="J8" s="72" t="s">
+        <v>102</v>
+      </c>
+      <c r="K8" s="72"/>
+      <c r="L8" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="M8" s="96" t="s">
+      <c r="M8" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="N8" s="96" t="s">
+      <c r="N8" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="O8" s="96" t="s">
-        <v>99</v>
-      </c>
-      <c r="P8" s="97">
+      <c r="O8" s="73" t="s">
+        <v>87</v>
+      </c>
+      <c r="P8" s="69">
         <v>0</v>
       </c>
-      <c r="Q8" s="97">
+      <c r="Q8" s="69">
         <v>1</v>
       </c>
-      <c r="R8" s="97">
+      <c r="R8" s="69">
         <v>2</v>
       </c>
-      <c r="S8" s="97" t="s">
+      <c r="S8" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="T8" s="97" t="s">
+      <c r="T8" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="U8" s="97" t="s">
+      <c r="U8" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="V8" s="97" t="s">
+      <c r="V8" s="69" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="2:22" ht="15.75">
-      <c r="B9" s="98"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="93"/>
-      <c r="E9" s="94"/>
+    <row r="9" spans="2:22" ht="17" x14ac:dyDescent="0.2">
+      <c r="B9" s="66"/>
+      <c r="C9" s="71"/>
+      <c r="D9" s="71"/>
+      <c r="E9" s="74"/>
       <c r="F9" s="9" t="s">
         <v>43</v>
       </c>
@@ -2728,30 +2761,30 @@
       <c r="K9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L9" s="96"/>
-      <c r="M9" s="96"/>
-      <c r="N9" s="96"/>
-      <c r="O9" s="96"/>
-      <c r="P9" s="97"/>
-      <c r="Q9" s="97"/>
-      <c r="R9" s="97"/>
-      <c r="S9" s="97"/>
-      <c r="T9" s="97"/>
-      <c r="U9" s="97"/>
-      <c r="V9" s="97"/>
-    </row>
-    <row r="10" spans="2:22" ht="15.75">
+      <c r="L9" s="73"/>
+      <c r="M9" s="73"/>
+      <c r="N9" s="73"/>
+      <c r="O9" s="73"/>
+      <c r="P9" s="69"/>
+      <c r="Q9" s="69"/>
+      <c r="R9" s="69"/>
+      <c r="S9" s="69"/>
+      <c r="T9" s="69"/>
+      <c r="U9" s="69"/>
+      <c r="V9" s="69"/>
+    </row>
+    <row r="10" spans="2:22" ht="17" x14ac:dyDescent="0.2">
       <c r="B10" s="10" t="s">
         <v>45</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="13" t="s">
@@ -2766,31 +2799,33 @@
         <v>44</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="M10" s="14"/>
       <c r="N10" s="14"/>
       <c r="O10" s="14"/>
       <c r="P10" s="15"/>
       <c r="Q10" s="15"/>
-      <c r="R10" s="15"/>
+      <c r="R10" s="15" t="s">
+        <v>103</v>
+      </c>
       <c r="S10" s="15"/>
       <c r="T10" s="15"/>
       <c r="U10" s="15"/>
       <c r="V10" s="15"/>
     </row>
-    <row r="11" spans="2:22" ht="30">
+    <row r="11" spans="2:22" ht="34" x14ac:dyDescent="0.2">
       <c r="B11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>43</v>
@@ -2806,30 +2841,32 @@
       <c r="K11" s="13"/>
       <c r="L11" s="14"/>
       <c r="M11" s="14" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="N11" s="14"/>
       <c r="O11" s="14"/>
       <c r="P11" s="15"/>
       <c r="Q11" s="15"/>
-      <c r="R11" s="15"/>
+      <c r="R11" s="15" t="s">
+        <v>103</v>
+      </c>
       <c r="S11" s="15"/>
       <c r="T11" s="15"/>
       <c r="U11" s="15"/>
       <c r="V11" s="15"/>
     </row>
-    <row r="12" spans="2:22" ht="31.5">
+    <row r="12" spans="2:22" ht="34" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>44</v>
@@ -2846,29 +2883,31 @@
       <c r="L12" s="14"/>
       <c r="M12" s="14"/>
       <c r="N12" s="14" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="O12" s="14"/>
       <c r="P12" s="15"/>
       <c r="Q12" s="15"/>
-      <c r="R12" s="15"/>
+      <c r="R12" s="15" t="s">
+        <v>103</v>
+      </c>
       <c r="S12" s="15"/>
       <c r="T12" s="15"/>
       <c r="U12" s="15"/>
       <c r="V12" s="15"/>
     </row>
-    <row r="13" spans="2:22" ht="30">
+    <row r="13" spans="2:22" ht="34" x14ac:dyDescent="0.2">
       <c r="B13" s="10" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>43</v>
@@ -2886,17 +2925,19 @@
       <c r="M13" s="14"/>
       <c r="N13" s="14"/>
       <c r="O13" s="14" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="P13" s="15"/>
       <c r="Q13" s="15"/>
-      <c r="R13" s="15"/>
+      <c r="R13" s="15" t="s">
+        <v>103</v>
+      </c>
       <c r="S13" s="15"/>
       <c r="T13" s="15"/>
       <c r="U13" s="15"/>
       <c r="V13" s="15"/>
     </row>
-    <row r="14" spans="2:22" ht="15.75">
+    <row r="14" spans="2:22" ht="17" x14ac:dyDescent="0.2">
       <c r="B14" s="10" t="s">
         <v>19</v>
       </c>
@@ -2921,7 +2962,7 @@
       <c r="U14" s="15"/>
       <c r="V14" s="15"/>
     </row>
-    <row r="15" spans="2:22" ht="15.75">
+    <row r="15" spans="2:22" ht="17" x14ac:dyDescent="0.2">
       <c r="B15" s="10" t="s">
         <v>19</v>
       </c>
@@ -2946,11 +2987,21 @@
       <c r="U15" s="15"/>
       <c r="V15" s="15"/>
     </row>
-    <row r="16" spans="2:22" ht="15.75">
+    <row r="16" spans="2:22" ht="16" x14ac:dyDescent="0.2">
       <c r="B16" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F7:K7"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
     <mergeCell ref="D1:G1"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B6:B9"/>
@@ -2967,16 +3018,6 @@
     <mergeCell ref="P7:V7"/>
     <mergeCell ref="V8:V9"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:K7"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="J8:K8"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2990,69 +3031,69 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:N16"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.796875" customWidth="1"/>
-    <col min="3" max="3" width="13.86328125" customWidth="1"/>
-    <col min="4" max="4" width="18.796875" customWidth="1"/>
-    <col min="5" max="6" width="16.1328125" customWidth="1"/>
-    <col min="7" max="7" width="55.3984375" customWidth="1"/>
-    <col min="8" max="8" width="58.3984375" customWidth="1"/>
-    <col min="10" max="10" width="7.1328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.1328125" customWidth="1"/>
-    <col min="13" max="13" width="16.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="6" width="16.1640625" customWidth="1"/>
+    <col min="7" max="7" width="55.33203125" customWidth="1"/>
+    <col min="8" max="8" width="58.33203125" customWidth="1"/>
+    <col min="10" max="10" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.1640625" customWidth="1"/>
+    <col min="13" max="13" width="16.1640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B1" s="8"/>
-      <c r="D1" s="61" t="s">
+      <c r="D1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="63"/>
-    </row>
-    <row r="3" spans="2:14">
-      <c r="B3" s="36" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="46"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B3" s="106" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="38"/>
-    </row>
-    <row r="4" spans="2:14">
-      <c r="B4" s="64" t="s">
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="108"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B4" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="56" t="s">
+      <c r="C4" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="D4" s="81" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="E4" s="103" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="35"/>
-      <c r="G4" s="34" t="s">
+      <c r="F4" s="104"/>
+      <c r="G4" s="105" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="35"/>
-    </row>
-    <row r="5" spans="2:14" ht="14.65" thickBot="1">
-      <c r="B5" s="65"/>
-      <c r="C5" s="68"/>
-      <c r="D5" s="70"/>
-      <c r="E5" s="101" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" s="102" t="s">
-        <v>121</v>
+      <c r="H4" s="104"/>
+    </row>
+    <row r="5" spans="2:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="76"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>52</v>
@@ -3061,97 +3102,97 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="2:14" ht="14.65" thickTop="1">
+    <row r="6" spans="2:14" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B6" s="19">
         <v>9</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="106">
+      <c r="E6" s="34">
         <v>1</v>
       </c>
-      <c r="F6" s="108">
+      <c r="F6" s="34">
         <v>5</v>
       </c>
-      <c r="G6" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="H6" s="109" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="2:14">
+      <c r="G6" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B7" s="19">
         <v>10</v>
       </c>
-      <c r="C7" s="66"/>
+      <c r="C7" s="77"/>
       <c r="D7" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="105">
+      <c r="E7" s="19">
         <v>0</v>
       </c>
-      <c r="F7" s="107">
+      <c r="F7" s="19">
         <v>2</v>
       </c>
-      <c r="G7" s="109" t="s">
-        <v>122</v>
-      </c>
-      <c r="H7" s="109" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="8" spans="2:14">
+      <c r="G7" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B8" s="19">
         <v>11</v>
       </c>
-      <c r="C8" s="66"/>
-      <c r="D8" s="103" t="s">
-        <v>106</v>
-      </c>
-      <c r="E8" s="105">
+      <c r="C8" s="77"/>
+      <c r="D8" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E8" s="19">
         <v>2</v>
       </c>
-      <c r="F8" s="107">
+      <c r="F8" s="19">
         <v>-1</v>
       </c>
-      <c r="G8" s="109" t="s">
-        <v>123</v>
-      </c>
-      <c r="H8" s="109" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="9" spans="2:14">
+      <c r="G8" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B9" s="19">
         <v>12</v>
       </c>
-      <c r="C9" s="66"/>
-      <c r="D9" s="104" t="s">
-        <v>107</v>
-      </c>
-      <c r="E9" s="105">
+      <c r="C9" s="77"/>
+      <c r="D9" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" s="19">
         <v>-3</v>
       </c>
-      <c r="F9" s="107">
+      <c r="F9" s="19">
         <v>0</v>
       </c>
-      <c r="G9" s="109" t="s">
-        <v>124</v>
-      </c>
-      <c r="H9" s="109" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14" ht="14.65" thickBot="1">
+      <c r="G9" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>13</v>
       </c>
-      <c r="C10" s="67"/>
+      <c r="C10" s="78"/>
       <c r="D10" s="6" t="s">
         <v>19</v>
       </c>
@@ -3168,7 +3209,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="2:14" ht="14.65" thickTop="1">
+    <row r="11" spans="2:14" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -3181,140 +3222,136 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
     </row>
-    <row r="12" spans="2:14" ht="14.65" thickBot="1">
+    <row r="12" spans="2:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>56</v>
       </c>
       <c r="K12" s="20"/>
     </row>
-    <row r="13" spans="2:14" ht="15" thickTop="1" thickBot="1">
-      <c r="B13" s="39" t="s">
+    <row r="13" spans="2:14" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="99" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="71" t="s">
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="101" t="s">
         <v>58</v>
       </c>
-      <c r="G13" s="72"/>
-      <c r="H13" s="39" t="s">
+      <c r="G13" s="102"/>
+      <c r="H13" s="99" t="s">
         <v>59</v>
       </c>
-      <c r="I13" s="40"/>
-      <c r="J13" s="40"/>
-      <c r="K13" s="40"/>
-      <c r="L13" s="41"/>
-      <c r="M13" s="46" t="s">
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="109"/>
+      <c r="M13" s="85" t="s">
         <v>60</v>
       </c>
-      <c r="N13" s="47"/>
-    </row>
-    <row r="14" spans="2:14" ht="14.65" thickTop="1">
-      <c r="B14" s="45" t="s">
+      <c r="N13" s="86"/>
+    </row>
+    <row r="14" spans="2:14" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="84" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="49" t="s">
+      <c r="C14" s="88" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="49" t="s">
+      <c r="D14" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="51" t="s">
+      <c r="E14" s="90" t="s">
         <v>64</v>
       </c>
-      <c r="F14" s="53" t="s">
+      <c r="F14" s="92" t="s">
         <v>65</v>
       </c>
-      <c r="G14" s="55" t="s">
+      <c r="G14" s="94" t="s">
         <v>66</v>
       </c>
-      <c r="H14" s="57" t="s">
+      <c r="H14" s="95" t="s">
         <v>67</v>
       </c>
-      <c r="I14" s="49" t="s">
+      <c r="I14" s="88" t="s">
         <v>61</v>
       </c>
-      <c r="J14" s="49" t="s">
+      <c r="J14" s="88" t="s">
         <v>62</v>
       </c>
-      <c r="K14" s="59" t="s">
+      <c r="K14" s="97" t="s">
         <v>68</v>
       </c>
-      <c r="L14" s="42" t="s">
+      <c r="L14" s="110" t="s">
         <v>69</v>
       </c>
-      <c r="M14" s="44" t="s">
+      <c r="M14" s="83" t="s">
         <v>70</v>
       </c>
-      <c r="N14" s="56" t="s">
+      <c r="N14" s="79" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:14">
-      <c r="B15" s="48"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="58"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="50"/>
-      <c r="K15" s="60"/>
-      <c r="L15" s="43"/>
-      <c r="M15" s="45"/>
-      <c r="N15" s="53"/>
-    </row>
-    <row r="16" spans="2:14">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B15" s="87"/>
+      <c r="C15" s="89"/>
+      <c r="D15" s="89"/>
+      <c r="E15" s="91"/>
+      <c r="F15" s="93"/>
+      <c r="G15" s="94"/>
+      <c r="H15" s="96"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="89"/>
+      <c r="K15" s="98"/>
+      <c r="L15" s="111"/>
+      <c r="M15" s="84"/>
+      <c r="N15" s="92"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B16" s="21">
         <f>SUM(C16:D16)</f>
         <v>4</v>
       </c>
-      <c r="C16" s="114">
+      <c r="C16" s="38">
         <v>4</v>
       </c>
-      <c r="D16" s="114">
+      <c r="D16" s="38">
         <v>0</v>
       </c>
-      <c r="E16" s="115">
+      <c r="E16" s="39">
         <v>100</v>
       </c>
-      <c r="F16" s="116">
+      <c r="F16" s="40">
         <v>0</v>
       </c>
-      <c r="G16" s="113">
+      <c r="G16" s="37">
         <v>0</v>
       </c>
-      <c r="H16" s="112">
+      <c r="H16" s="36">
         <v>0</v>
       </c>
-      <c r="I16" s="117">
+      <c r="I16" s="21">
         <v>4</v>
       </c>
-      <c r="J16" s="114">
+      <c r="J16" s="38">
         <v>4</v>
       </c>
-      <c r="K16" s="118">
+      <c r="K16" s="41">
         <v>0</v>
       </c>
-      <c r="L16" s="119">
+      <c r="L16" s="42">
         <v>100</v>
       </c>
-      <c r="M16" s="111" t="s">
+      <c r="M16" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="N16" s="120" t="s">
-        <v>125</v>
+      <c r="N16" s="43" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C6:C10"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="L14:L15"/>
     <mergeCell ref="M14:M15"/>
     <mergeCell ref="M13:N13"/>
     <mergeCell ref="B14:B15"/>
@@ -3330,11 +3367,15 @@
     <mergeCell ref="J14:J15"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C6:C10"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="B3:H3"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="L14:L15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3342,14 +3383,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="301f98df-4edd-4096-94f8-2f8af3eee570">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3542,21 +3581,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="301f98df-4edd-4096-94f8-2f8af3eee570">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2F5940-EC19-4D08-A8C2-FA31EF734077}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EECFCB93-350B-4228-B7F4-DB12383611F2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="301f98df-4edd-4096-94f8-2f8af3eee570"/>
-    <ds:schemaRef ds:uri="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3581,9 +3619,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EECFCB93-350B-4228-B7F4-DB12383611F2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2F5940-EC19-4D08-A8C2-FA31EF734077}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="301f98df-4edd-4096-94f8-2f8af3eee570"/>
+    <ds:schemaRef ds:uri="cbfc0213-1ef7-4e52-9599-c30bc1b3f3d7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>